<commit_message>
modif super nutri score
</commit_message>
<xml_diff>
--- a/outputs/excel/dataset_avec_preds.xlsx
+++ b/outputs/excel/dataset_avec_preds.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T26"/>
+  <dimension ref="A1:Y26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,31 @@
           <t>electre_cat</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>is_bio</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>green_points</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>electre_points</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>super_score</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>super_label</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -613,6 +638,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -697,6 +739,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -781,6 +840,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -865,6 +941,23 @@
           <t>B'</t>
         </is>
       </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.8999999999999999</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -949,6 +1042,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1033,6 +1143,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1117,6 +1244,23 @@
           <t>B'</t>
         </is>
       </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" t="n">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0.8999999999999999</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1201,6 +1345,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1285,6 +1446,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1369,6 +1547,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1453,6 +1648,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1537,6 +1749,23 @@
           <t>B'</t>
         </is>
       </c>
+      <c r="U13" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" t="n">
+        <v>1</v>
+      </c>
+      <c r="W13" t="n">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1621,6 +1850,23 @@
           <t>B'</t>
         </is>
       </c>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1</v>
+      </c>
+      <c r="W14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1705,6 +1951,23 @@
           <t>B'</t>
         </is>
       </c>
+      <c r="U15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W15" t="n">
+        <v>1</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1789,6 +2052,23 @@
           <t>A'</t>
         </is>
       </c>
+      <c r="U16" t="n">
+        <v>1</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1</v>
+      </c>
+      <c r="W16" t="n">
+        <v>2</v>
+      </c>
+      <c r="X16" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1873,6 +2153,23 @@
           <t>D'</t>
         </is>
       </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
+        <v>-2</v>
+      </c>
+      <c r="W17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1957,6 +2254,23 @@
           <t>D'</t>
         </is>
       </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>-2</v>
+      </c>
+      <c r="W18" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X18" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2041,6 +2355,23 @@
           <t>D'</t>
         </is>
       </c>
+      <c r="U19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" t="n">
+        <v>-2</v>
+      </c>
+      <c r="W19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X19" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2125,6 +2456,23 @@
           <t>D'</t>
         </is>
       </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>-2</v>
+      </c>
+      <c r="W20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X20" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2209,6 +2557,23 @@
           <t>D'</t>
         </is>
       </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" t="n">
+        <v>1</v>
+      </c>
+      <c r="W21" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X21" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2293,6 +2658,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="n">
+        <v>1</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2377,6 +2759,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U23" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" t="n">
+        <v>1</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2461,6 +2860,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U24" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>1</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2545,6 +2961,23 @@
           <t>C'</t>
         </is>
       </c>
+      <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
+        <v>1</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2627,6 +3060,23 @@
       <c r="T26" t="inlineStr">
         <is>
           <t>C'</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" t="n">
+        <v>1</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>

</xml_diff>